<commit_message>
Agrega sesión 11 de reposición con laboratorio individual
</commit_message>
<xml_diff>
--- a/laboratorios/sesion09/laboratorio_dinero_inflacion.xlsx
+++ b/laboratorios/sesion09/laboratorio_dinero_inflacion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/paulogarridogrijalva/Documents/Docencia/2026/III/Macroeconomía/macroeconomia-200fp/laboratorios/sesion09/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4695174-9454-644F-AA61-57B778F0AE40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8159990E-0A2B-7E41-A522-87CC91B6F294}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Proyecto" sheetId="1" r:id="rId1"/>
@@ -281,13 +281,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="8">
+    <numFmt numFmtId="8" formatCode="&quot;Q&quot;#,##0.00;[Red]\-&quot;Q&quot;#,##0.00"/>
     <numFmt numFmtId="164" formatCode="&quot;Q&quot;\ #,##0;\(&quot;Q&quot;\ #,##0\);&quot;–&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
-    <numFmt numFmtId="168" formatCode="0.00&quot; x&quot;"/>
-    <numFmt numFmtId="169" formatCode="&quot;Q&quot;\ #,##0.00"/>
-    <numFmt numFmtId="170" formatCode="&quot;Q&quot;\ #,##0.00;\(&quot;Q&quot;\ #,##0.00\);&quot;Q 0.00&quot;"/>
+    <numFmt numFmtId="167" formatCode="0.00&quot; x&quot;"/>
+    <numFmt numFmtId="168" formatCode="&quot;Q&quot;\ #,##0.00"/>
+    <numFmt numFmtId="169" formatCode="&quot;Q&quot;\ #,##0.00;\(&quot;Q&quot;\ #,##0.00\);&quot;Q 0.00&quot;"/>
+    <numFmt numFmtId="170" formatCode="&quot;Q&quot;#,##0.00"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -381,7 +383,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -426,7 +428,7 @@
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -435,20 +437,24 @@
     <xf numFmtId="164" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="3" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="170" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -667,12 +673,13 @@
   <sheetPr>
     <tabColor rgb="FF0B2E4F"/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="43" customWidth="1"/>
     <col min="3" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25" customHeight="1">
@@ -711,7 +718,7 @@
       </c>
       <c r="C4" s="3">
         <f>SUM(C32:G32)-C12</f>
-        <v>794168.02966247033</v>
+        <v>760437.96790719032</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
@@ -725,7 +732,7 @@
       </c>
       <c r="C5" s="3">
         <f>SUM(C35:G35)-C12</f>
-        <v>794168.02966247033</v>
+        <v>760437.96790719032</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
@@ -862,7 +869,7 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" spans="1:7" ht="25" customHeight="1">
+    <row r="17" spans="1:8" ht="25" customHeight="1">
       <c r="A17" s="1"/>
       <c r="B17" s="2" t="s">
         <v>12</v>
@@ -875,7 +882,7 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:7" ht="25" customHeight="1">
+    <row r="18" spans="1:8" ht="25" customHeight="1">
       <c r="A18" s="1"/>
       <c r="B18" s="2" t="s">
         <v>13</v>
@@ -888,7 +895,7 @@
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
     </row>
-    <row r="19" spans="1:7" ht="25" customHeight="1">
+    <row r="19" spans="1:8" ht="25" customHeight="1">
       <c r="A19" s="1"/>
       <c r="B19" s="2" t="s">
         <v>14</v>
@@ -902,7 +909,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
     </row>
-    <row r="20" spans="1:7" ht="25" customHeight="1">
+    <row r="20" spans="1:8" ht="25" customHeight="1">
       <c r="A20" s="1"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -911,7 +918,7 @@
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
     </row>
-    <row r="21" spans="1:7" ht="29" customHeight="1">
+    <row r="21" spans="1:8" ht="29" customHeight="1">
       <c r="A21" s="1"/>
       <c r="B21" s="4" t="s">
         <v>15</v>
@@ -932,16 +939,16 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="25" customHeight="1">
+    <row r="22" spans="1:8" ht="25" customHeight="1">
       <c r="A22" s="1"/>
       <c r="B22" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C22" s="8">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="D22" s="8">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E22" s="8">
         <v>0.04</v>
@@ -953,16 +960,16 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="25" customHeight="1">
+    <row r="23" spans="1:8" ht="25" customHeight="1">
       <c r="A23" s="1"/>
       <c r="B23" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C23" s="8">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="D23" s="8">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E23" s="8">
         <v>0.04</v>
@@ -974,16 +981,16 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="25" customHeight="1">
+    <row r="24" spans="1:8" ht="25" customHeight="1">
       <c r="A24" s="1"/>
       <c r="B24" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C24" s="8">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="D24" s="8">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E24" s="8">
         <v>0.04</v>
@@ -995,16 +1002,16 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="25" customHeight="1">
+    <row r="25" spans="1:8" ht="25" customHeight="1">
       <c r="A25" s="1"/>
       <c r="B25" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C25" s="8">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="D25" s="8">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E25" s="8">
         <v>0.04</v>
@@ -1016,7 +1023,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="25" customHeight="1">
+    <row r="26" spans="1:8" ht="25" customHeight="1">
       <c r="A26" s="1"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -1025,160 +1032,161 @@
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
     </row>
-    <row r="27" spans="1:7" ht="25" customHeight="1">
+    <row r="27" spans="1:8" ht="25" customHeight="1">
       <c r="A27" s="1"/>
       <c r="B27" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C27" s="10">
         <f>1+C22</f>
-        <v>1.04</v>
+        <v>1.08</v>
       </c>
       <c r="D27" s="10">
         <f t="shared" ref="D27:G30" si="0">C27*(1+D22)</f>
-        <v>1.0816000000000001</v>
+        <v>1.1664000000000001</v>
       </c>
       <c r="E27" s="10">
         <f t="shared" si="0"/>
-        <v>1.1248640000000001</v>
+        <v>1.2130560000000001</v>
       </c>
       <c r="F27" s="10">
         <f t="shared" si="0"/>
-        <v>1.1698585600000002</v>
+        <v>1.2615782400000002</v>
       </c>
       <c r="G27" s="10">
         <f t="shared" si="0"/>
-        <v>1.2166529024000003</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="25" customHeight="1">
+        <v>1.3120413696000002</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="25" customHeight="1">
       <c r="A28" s="1"/>
       <c r="B28" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C28" s="21">
         <f>$C$14*(1+C23)</f>
-        <v>31.200000000000003</v>
+        <v>32.400000000000006</v>
       </c>
       <c r="D28" s="21">
         <f t="shared" si="0"/>
-        <v>32.448000000000008</v>
+        <v>34.992000000000012</v>
       </c>
       <c r="E28" s="21">
         <f t="shared" si="0"/>
-        <v>33.745920000000012</v>
+        <v>36.391680000000015</v>
       </c>
       <c r="F28" s="21">
         <f t="shared" si="0"/>
-        <v>35.095756800000011</v>
+        <v>37.847347200000016</v>
       </c>
       <c r="G28" s="21">
         <f t="shared" si="0"/>
-        <v>36.499587072000011</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="25" customHeight="1">
+        <v>39.361241088000021</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="25" customHeight="1">
       <c r="A29" s="1"/>
       <c r="B29" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C29" s="21">
         <f>$C$15*(1+C24)</f>
-        <v>18.72</v>
+        <v>19.8</v>
       </c>
       <c r="D29" s="21">
         <f t="shared" si="0"/>
-        <v>19.468799999999998</v>
+        <v>21.78</v>
       </c>
       <c r="E29" s="21">
         <f t="shared" si="0"/>
-        <v>20.247551999999999</v>
+        <v>22.651200000000003</v>
       </c>
       <c r="F29" s="21">
         <f t="shared" si="0"/>
-        <v>21.057454079999999</v>
+        <v>23.557248000000005</v>
       </c>
       <c r="G29" s="21">
         <f t="shared" si="0"/>
-        <v>21.899752243200002</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="25" customHeight="1">
+        <v>24.499537920000005</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="25" customHeight="1">
       <c r="A30" s="1"/>
       <c r="B30" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C30" s="3">
         <f>$C$16*(1+C25)</f>
-        <v>416000</v>
+        <v>432000</v>
       </c>
       <c r="D30" s="3">
         <f t="shared" si="0"/>
-        <v>432640</v>
+        <v>466560.00000000006</v>
       </c>
       <c r="E30" s="3">
         <f t="shared" si="0"/>
-        <v>449945.60000000003</v>
+        <v>485222.40000000008</v>
       </c>
       <c r="F30" s="3">
         <f t="shared" si="0"/>
-        <v>467943.42400000006</v>
+        <v>504631.29600000009</v>
       </c>
       <c r="G30" s="3">
         <f t="shared" si="0"/>
-        <v>486661.16096000007</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="25" customHeight="1">
+        <v>524816.54784000013</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="25" customHeight="1">
       <c r="A31" s="1"/>
       <c r="B31" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C31" s="12">
         <f>$C$13*(C28-C29)-C30</f>
-        <v>832000.00000000047</v>
+        <v>828000.00000000047</v>
       </c>
       <c r="D31" s="12">
         <f>$C$13*(D28-D29)-D30</f>
-        <v>865280.00000000093</v>
+        <v>854640.00000000093</v>
       </c>
       <c r="E31" s="12">
         <f>$C$13*(E28-E29)-E30</f>
-        <v>899891.20000000135</v>
+        <v>888825.60000000102</v>
       </c>
       <c r="F31" s="12">
         <f>$C$13*(F28-F29)-F30</f>
-        <v>935886.84800000093</v>
+        <v>924378.624000001</v>
       </c>
       <c r="G31" s="12">
         <f>$C$13*(G28-G29)-G30</f>
-        <v>973322.32192000095</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="25" customHeight="1">
+        <v>961353.76896000141</v>
+      </c>
+      <c r="H31" s="25"/>
+    </row>
+    <row r="32" spans="1:8" ht="25" customHeight="1">
       <c r="A32" s="1"/>
       <c r="B32" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C32" s="3">
         <f>C31/(1+$C$19)^C$21</f>
-        <v>740740.74074074102</v>
+        <v>737179.48717948748</v>
       </c>
       <c r="D32" s="3">
         <f>D31/(1+$C$19)^D$21</f>
-        <v>685871.05624142708</v>
+        <v>677437.17583461222</v>
       </c>
       <c r="E32" s="3">
         <f>E31/(1+$C$19)^E$21</f>
-        <v>635065.79281613638</v>
+        <v>627256.64429130754</v>
       </c>
       <c r="F32" s="3">
         <f>F31/(1+$C$19)^F$21</f>
-        <v>588023.88223716291</v>
+        <v>580793.18915861798</v>
       </c>
       <c r="G32" s="3">
         <f>G31/(1+$C$19)^G$21</f>
-        <v>544466.55762700259</v>
+        <v>537771.47144316486</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="25" customHeight="1">
@@ -1188,23 +1196,23 @@
       </c>
       <c r="C33" s="3">
         <f>C31/C27</f>
-        <v>800000.00000000047</v>
+        <v>766666.66666666709</v>
       </c>
       <c r="D33" s="3">
         <f>D31/D27</f>
-        <v>800000.00000000081</v>
+        <v>732716.04938271677</v>
       </c>
       <c r="E33" s="3">
         <f>E31/E27</f>
-        <v>800000.00000000116</v>
+        <v>732716.04938271677</v>
       </c>
       <c r="F33" s="3">
         <f>F31/F27</f>
-        <v>800000.0000000007</v>
+        <v>732716.04938271677</v>
       </c>
       <c r="G33" s="3">
         <f>G31/G27</f>
-        <v>800000.00000000058</v>
+        <v>732716.049382717</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="25" customHeight="1">
@@ -1214,23 +1222,23 @@
       </c>
       <c r="C34" s="10">
         <f>(1+$C$19)^C$21/C27</f>
-        <v>1.08</v>
+        <v>1.04</v>
       </c>
       <c r="D34" s="10">
         <f>(1+$C$19)^D$21/D27</f>
-        <v>1.1664000000000003</v>
+        <v>1.0816000000000003</v>
       </c>
       <c r="E34" s="10">
         <f>(1+$C$19)^E$21/E27</f>
-        <v>1.2597120000000004</v>
+        <v>1.1681280000000005</v>
       </c>
       <c r="F34" s="10">
         <f>(1+$C$19)^F$21/F27</f>
-        <v>1.3604889600000007</v>
+        <v>1.2615782400000006</v>
       </c>
       <c r="G34" s="10">
         <f>(1+$C$19)^G$21/G27</f>
-        <v>1.4693280768000008</v>
+        <v>1.3625044992000011</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="25" customHeight="1">
@@ -1240,33 +1248,33 @@
       </c>
       <c r="C35" s="12">
         <f>C33/C34</f>
-        <v>740740.74074074114</v>
+        <v>737179.48717948759</v>
       </c>
       <c r="D35" s="12">
         <f>D33/D34</f>
-        <v>685871.05624142708</v>
+        <v>677437.17583461222</v>
       </c>
       <c r="E35" s="12">
         <f>E33/E34</f>
-        <v>635065.7928161365</v>
+        <v>627256.64429130754</v>
       </c>
       <c r="F35" s="12">
         <f>F33/F34</f>
-        <v>588023.88223716291</v>
+        <v>580793.18915861798</v>
       </c>
       <c r="G35" s="12">
         <f>G33/G34</f>
-        <v>544466.55762700259</v>
+        <v>537771.47144316486</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="25" customHeight="1">
       <c r="A36" s="1"/>
       <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
+      <c r="C36" s="26"/>
+      <c r="D36" s="26"/>
+      <c r="E36" s="26"/>
+      <c r="F36" s="26"/>
+      <c r="G36" s="26"/>
     </row>
     <row r="37" spans="1:7" ht="25" customHeight="1">
       <c r="A37" s="1"/>
@@ -1478,7 +1486,10 @@
       <c r="B10" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="15"/>
+      <c r="C10" s="15">
+        <f>C6+C7*C8*C9</f>
+        <v>0.11</v>
+      </c>
       <c r="D10" s="15"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -1573,23 +1584,23 @@
       </c>
       <c r="C15" s="3">
         <f>C13*$C$10</f>
-        <v>0</v>
+        <v>132000</v>
       </c>
       <c r="D15" s="3">
         <f>D13*$C$10</f>
-        <v>0</v>
+        <v>105600</v>
       </c>
       <c r="E15" s="3">
         <f>E13*$C$10</f>
-        <v>0</v>
+        <v>79200</v>
       </c>
       <c r="F15" s="3">
         <f>F13*$C$10</f>
-        <v>0</v>
+        <v>52800</v>
       </c>
       <c r="G15" s="3">
         <f>G13*$C$10</f>
-        <v>0</v>
+        <v>26400</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="25" customHeight="1">
@@ -1599,23 +1610,23 @@
       </c>
       <c r="C16" s="3">
         <f>C14+C15</f>
-        <v>240000</v>
+        <v>372000</v>
       </c>
       <c r="D16" s="3">
         <f>D14+D15</f>
-        <v>240000</v>
+        <v>345600</v>
       </c>
       <c r="E16" s="3">
         <f>E14+E15</f>
-        <v>240000</v>
+        <v>319200</v>
       </c>
       <c r="F16" s="3">
         <f>F14+F15</f>
-        <v>240000</v>
+        <v>292800</v>
       </c>
       <c r="G16" s="3">
         <f>G14+G15</f>
-        <v>240000</v>
+        <v>266400</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="25" customHeight="1">
@@ -1660,23 +1671,23 @@
       </c>
       <c r="C19" s="17">
         <f>Proyecto!C31</f>
-        <v>832000.00000000047</v>
+        <v>828000.00000000047</v>
       </c>
       <c r="D19" s="17">
         <f>Proyecto!D31</f>
-        <v>865280.00000000093</v>
+        <v>854640.00000000093</v>
       </c>
       <c r="E19" s="17">
         <f>Proyecto!E31</f>
-        <v>899891.20000000135</v>
+        <v>888825.60000000102</v>
       </c>
       <c r="F19" s="17">
         <f>Proyecto!F31</f>
-        <v>935886.84800000093</v>
+        <v>924378.624000001</v>
       </c>
       <c r="G19" s="17">
         <f>Proyecto!G31</f>
-        <v>973322.32192000095</v>
+        <v>961353.76896000141</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="25" customHeight="1">
@@ -1686,23 +1697,23 @@
       </c>
       <c r="C20" s="16">
         <f>IF(C16=0,"Sin deuda",C19/C16)</f>
-        <v>3.4666666666666686</v>
+        <v>2.2258064516129044</v>
       </c>
       <c r="D20" s="16">
         <f>IF(D16=0,"Sin deuda",D19/D16)</f>
-        <v>3.6053333333333373</v>
+        <v>2.4729166666666695</v>
       </c>
       <c r="E20" s="16">
         <f>IF(E16=0,"Sin deuda",E19/E16)</f>
-        <v>3.7495466666666721</v>
+        <v>2.784541353383462</v>
       </c>
       <c r="F20" s="16">
         <f>IF(F16=0,"Sin deuda",F19/F16)</f>
-        <v>3.8995285333333372</v>
+        <v>3.1570308196721344</v>
       </c>
       <c r="G20" s="16">
         <f>IF(G16=0,"Sin deuda",G19/G16)</f>
-        <v>4.0555096746666708</v>
+        <v>3.6086853189189241</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="25" customHeight="1">
@@ -1712,23 +1723,23 @@
       </c>
       <c r="C21" s="3">
         <f>C19-C16</f>
-        <v>592000.00000000047</v>
+        <v>456000.00000000047</v>
       </c>
       <c r="D21" s="3">
         <f>D19-D16</f>
-        <v>625280.00000000093</v>
+        <v>509040.00000000093</v>
       </c>
       <c r="E21" s="3">
         <f>E19-E16</f>
-        <v>659891.20000000135</v>
+        <v>569625.60000000102</v>
       </c>
       <c r="F21" s="3">
         <f>F19-F16</f>
-        <v>695886.84800000093</v>
+        <v>631578.624000001</v>
       </c>
       <c r="G21" s="3">
         <f>G19-G16</f>
-        <v>733322.32192000095</v>
+        <v>694953.76896000141</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="25" customHeight="1">
@@ -1876,8 +1887,8 @@
     </row>
     <row r="4" spans="1:7" ht="25" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="2" t="s">
-        <v>56</v>
+      <c r="B4" s="2" t="str">
+        <v>Trabajo individual: 45 minutos + discusión.</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -1966,8 +1977,8 @@
     </row>
     <row r="13" spans="1:7" ht="29" customHeight="1">
       <c r="A13" s="1"/>
-      <c r="B13" s="4" t="s">
-        <v>61</v>
+      <c r="B13" s="4" t="str">
+        <v>Registro individual</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>62</v>

</xml_diff>

<commit_message>
Publica sesión 11 y laboratorio individual
</commit_message>
<xml_diff>
--- a/laboratorios/sesion09/laboratorio_dinero_inflacion.xlsx
+++ b/laboratorios/sesion09/laboratorio_dinero_inflacion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/paulogarridogrijalva/Documents/Docencia/2026/III/Macroeconomía/macroeconomia-200fp/laboratorios/sesion09/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4695174-9454-644F-AA61-57B778F0AE40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8159990E-0A2B-7E41-A522-87CC91B6F294}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Proyecto" sheetId="1" r:id="rId1"/>
@@ -281,13 +281,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="8">
+    <numFmt numFmtId="8" formatCode="&quot;Q&quot;#,##0.00;[Red]\-&quot;Q&quot;#,##0.00"/>
     <numFmt numFmtId="164" formatCode="&quot;Q&quot;\ #,##0;\(&quot;Q&quot;\ #,##0\);&quot;–&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
-    <numFmt numFmtId="168" formatCode="0.00&quot; x&quot;"/>
-    <numFmt numFmtId="169" formatCode="&quot;Q&quot;\ #,##0.00"/>
-    <numFmt numFmtId="170" formatCode="&quot;Q&quot;\ #,##0.00;\(&quot;Q&quot;\ #,##0.00\);&quot;Q 0.00&quot;"/>
+    <numFmt numFmtId="167" formatCode="0.00&quot; x&quot;"/>
+    <numFmt numFmtId="168" formatCode="&quot;Q&quot;\ #,##0.00"/>
+    <numFmt numFmtId="169" formatCode="&quot;Q&quot;\ #,##0.00;\(&quot;Q&quot;\ #,##0.00\);&quot;Q 0.00&quot;"/>
+    <numFmt numFmtId="170" formatCode="&quot;Q&quot;#,##0.00"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -381,7 +383,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -426,7 +428,7 @@
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -435,20 +437,24 @@
     <xf numFmtId="164" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="3" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="170" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -667,12 +673,13 @@
   <sheetPr>
     <tabColor rgb="FF0B2E4F"/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="43" customWidth="1"/>
     <col min="3" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25" customHeight="1">
@@ -711,7 +718,7 @@
       </c>
       <c r="C4" s="3">
         <f>SUM(C32:G32)-C12</f>
-        <v>794168.02966247033</v>
+        <v>760437.96790719032</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
@@ -725,7 +732,7 @@
       </c>
       <c r="C5" s="3">
         <f>SUM(C35:G35)-C12</f>
-        <v>794168.02966247033</v>
+        <v>760437.96790719032</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
@@ -862,7 +869,7 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" spans="1:7" ht="25" customHeight="1">
+    <row r="17" spans="1:8" ht="25" customHeight="1">
       <c r="A17" s="1"/>
       <c r="B17" s="2" t="s">
         <v>12</v>
@@ -875,7 +882,7 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:7" ht="25" customHeight="1">
+    <row r="18" spans="1:8" ht="25" customHeight="1">
       <c r="A18" s="1"/>
       <c r="B18" s="2" t="s">
         <v>13</v>
@@ -888,7 +895,7 @@
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
     </row>
-    <row r="19" spans="1:7" ht="25" customHeight="1">
+    <row r="19" spans="1:8" ht="25" customHeight="1">
       <c r="A19" s="1"/>
       <c r="B19" s="2" t="s">
         <v>14</v>
@@ -902,7 +909,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
     </row>
-    <row r="20" spans="1:7" ht="25" customHeight="1">
+    <row r="20" spans="1:8" ht="25" customHeight="1">
       <c r="A20" s="1"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -911,7 +918,7 @@
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
     </row>
-    <row r="21" spans="1:7" ht="29" customHeight="1">
+    <row r="21" spans="1:8" ht="29" customHeight="1">
       <c r="A21" s="1"/>
       <c r="B21" s="4" t="s">
         <v>15</v>
@@ -932,16 +939,16 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="25" customHeight="1">
+    <row r="22" spans="1:8" ht="25" customHeight="1">
       <c r="A22" s="1"/>
       <c r="B22" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C22" s="8">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="D22" s="8">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E22" s="8">
         <v>0.04</v>
@@ -953,16 +960,16 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="25" customHeight="1">
+    <row r="23" spans="1:8" ht="25" customHeight="1">
       <c r="A23" s="1"/>
       <c r="B23" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C23" s="8">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="D23" s="8">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E23" s="8">
         <v>0.04</v>
@@ -974,16 +981,16 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="25" customHeight="1">
+    <row r="24" spans="1:8" ht="25" customHeight="1">
       <c r="A24" s="1"/>
       <c r="B24" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C24" s="8">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="D24" s="8">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E24" s="8">
         <v>0.04</v>
@@ -995,16 +1002,16 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="25" customHeight="1">
+    <row r="25" spans="1:8" ht="25" customHeight="1">
       <c r="A25" s="1"/>
       <c r="B25" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C25" s="8">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="D25" s="8">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="E25" s="8">
         <v>0.04</v>
@@ -1016,7 +1023,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="25" customHeight="1">
+    <row r="26" spans="1:8" ht="25" customHeight="1">
       <c r="A26" s="1"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -1025,160 +1032,161 @@
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
     </row>
-    <row r="27" spans="1:7" ht="25" customHeight="1">
+    <row r="27" spans="1:8" ht="25" customHeight="1">
       <c r="A27" s="1"/>
       <c r="B27" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C27" s="10">
         <f>1+C22</f>
-        <v>1.04</v>
+        <v>1.08</v>
       </c>
       <c r="D27" s="10">
         <f t="shared" ref="D27:G30" si="0">C27*(1+D22)</f>
-        <v>1.0816000000000001</v>
+        <v>1.1664000000000001</v>
       </c>
       <c r="E27" s="10">
         <f t="shared" si="0"/>
-        <v>1.1248640000000001</v>
+        <v>1.2130560000000001</v>
       </c>
       <c r="F27" s="10">
         <f t="shared" si="0"/>
-        <v>1.1698585600000002</v>
+        <v>1.2615782400000002</v>
       </c>
       <c r="G27" s="10">
         <f t="shared" si="0"/>
-        <v>1.2166529024000003</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="25" customHeight="1">
+        <v>1.3120413696000002</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="25" customHeight="1">
       <c r="A28" s="1"/>
       <c r="B28" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C28" s="21">
         <f>$C$14*(1+C23)</f>
-        <v>31.200000000000003</v>
+        <v>32.400000000000006</v>
       </c>
       <c r="D28" s="21">
         <f t="shared" si="0"/>
-        <v>32.448000000000008</v>
+        <v>34.992000000000012</v>
       </c>
       <c r="E28" s="21">
         <f t="shared" si="0"/>
-        <v>33.745920000000012</v>
+        <v>36.391680000000015</v>
       </c>
       <c r="F28" s="21">
         <f t="shared" si="0"/>
-        <v>35.095756800000011</v>
+        <v>37.847347200000016</v>
       </c>
       <c r="G28" s="21">
         <f t="shared" si="0"/>
-        <v>36.499587072000011</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="25" customHeight="1">
+        <v>39.361241088000021</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="25" customHeight="1">
       <c r="A29" s="1"/>
       <c r="B29" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C29" s="21">
         <f>$C$15*(1+C24)</f>
-        <v>18.72</v>
+        <v>19.8</v>
       </c>
       <c r="D29" s="21">
         <f t="shared" si="0"/>
-        <v>19.468799999999998</v>
+        <v>21.78</v>
       </c>
       <c r="E29" s="21">
         <f t="shared" si="0"/>
-        <v>20.247551999999999</v>
+        <v>22.651200000000003</v>
       </c>
       <c r="F29" s="21">
         <f t="shared" si="0"/>
-        <v>21.057454079999999</v>
+        <v>23.557248000000005</v>
       </c>
       <c r="G29" s="21">
         <f t="shared" si="0"/>
-        <v>21.899752243200002</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="25" customHeight="1">
+        <v>24.499537920000005</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="25" customHeight="1">
       <c r="A30" s="1"/>
       <c r="B30" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C30" s="3">
         <f>$C$16*(1+C25)</f>
-        <v>416000</v>
+        <v>432000</v>
       </c>
       <c r="D30" s="3">
         <f t="shared" si="0"/>
-        <v>432640</v>
+        <v>466560.00000000006</v>
       </c>
       <c r="E30" s="3">
         <f t="shared" si="0"/>
-        <v>449945.60000000003</v>
+        <v>485222.40000000008</v>
       </c>
       <c r="F30" s="3">
         <f t="shared" si="0"/>
-        <v>467943.42400000006</v>
+        <v>504631.29600000009</v>
       </c>
       <c r="G30" s="3">
         <f t="shared" si="0"/>
-        <v>486661.16096000007</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="25" customHeight="1">
+        <v>524816.54784000013</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="25" customHeight="1">
       <c r="A31" s="1"/>
       <c r="B31" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C31" s="12">
         <f>$C$13*(C28-C29)-C30</f>
-        <v>832000.00000000047</v>
+        <v>828000.00000000047</v>
       </c>
       <c r="D31" s="12">
         <f>$C$13*(D28-D29)-D30</f>
-        <v>865280.00000000093</v>
+        <v>854640.00000000093</v>
       </c>
       <c r="E31" s="12">
         <f>$C$13*(E28-E29)-E30</f>
-        <v>899891.20000000135</v>
+        <v>888825.60000000102</v>
       </c>
       <c r="F31" s="12">
         <f>$C$13*(F28-F29)-F30</f>
-        <v>935886.84800000093</v>
+        <v>924378.624000001</v>
       </c>
       <c r="G31" s="12">
         <f>$C$13*(G28-G29)-G30</f>
-        <v>973322.32192000095</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="25" customHeight="1">
+        <v>961353.76896000141</v>
+      </c>
+      <c r="H31" s="25"/>
+    </row>
+    <row r="32" spans="1:8" ht="25" customHeight="1">
       <c r="A32" s="1"/>
       <c r="B32" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C32" s="3">
         <f>C31/(1+$C$19)^C$21</f>
-        <v>740740.74074074102</v>
+        <v>737179.48717948748</v>
       </c>
       <c r="D32" s="3">
         <f>D31/(1+$C$19)^D$21</f>
-        <v>685871.05624142708</v>
+        <v>677437.17583461222</v>
       </c>
       <c r="E32" s="3">
         <f>E31/(1+$C$19)^E$21</f>
-        <v>635065.79281613638</v>
+        <v>627256.64429130754</v>
       </c>
       <c r="F32" s="3">
         <f>F31/(1+$C$19)^F$21</f>
-        <v>588023.88223716291</v>
+        <v>580793.18915861798</v>
       </c>
       <c r="G32" s="3">
         <f>G31/(1+$C$19)^G$21</f>
-        <v>544466.55762700259</v>
+        <v>537771.47144316486</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="25" customHeight="1">
@@ -1188,23 +1196,23 @@
       </c>
       <c r="C33" s="3">
         <f>C31/C27</f>
-        <v>800000.00000000047</v>
+        <v>766666.66666666709</v>
       </c>
       <c r="D33" s="3">
         <f>D31/D27</f>
-        <v>800000.00000000081</v>
+        <v>732716.04938271677</v>
       </c>
       <c r="E33" s="3">
         <f>E31/E27</f>
-        <v>800000.00000000116</v>
+        <v>732716.04938271677</v>
       </c>
       <c r="F33" s="3">
         <f>F31/F27</f>
-        <v>800000.0000000007</v>
+        <v>732716.04938271677</v>
       </c>
       <c r="G33" s="3">
         <f>G31/G27</f>
-        <v>800000.00000000058</v>
+        <v>732716.049382717</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="25" customHeight="1">
@@ -1214,23 +1222,23 @@
       </c>
       <c r="C34" s="10">
         <f>(1+$C$19)^C$21/C27</f>
-        <v>1.08</v>
+        <v>1.04</v>
       </c>
       <c r="D34" s="10">
         <f>(1+$C$19)^D$21/D27</f>
-        <v>1.1664000000000003</v>
+        <v>1.0816000000000003</v>
       </c>
       <c r="E34" s="10">
         <f>(1+$C$19)^E$21/E27</f>
-        <v>1.2597120000000004</v>
+        <v>1.1681280000000005</v>
       </c>
       <c r="F34" s="10">
         <f>(1+$C$19)^F$21/F27</f>
-        <v>1.3604889600000007</v>
+        <v>1.2615782400000006</v>
       </c>
       <c r="G34" s="10">
         <f>(1+$C$19)^G$21/G27</f>
-        <v>1.4693280768000008</v>
+        <v>1.3625044992000011</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="25" customHeight="1">
@@ -1240,33 +1248,33 @@
       </c>
       <c r="C35" s="12">
         <f>C33/C34</f>
-        <v>740740.74074074114</v>
+        <v>737179.48717948759</v>
       </c>
       <c r="D35" s="12">
         <f>D33/D34</f>
-        <v>685871.05624142708</v>
+        <v>677437.17583461222</v>
       </c>
       <c r="E35" s="12">
         <f>E33/E34</f>
-        <v>635065.7928161365</v>
+        <v>627256.64429130754</v>
       </c>
       <c r="F35" s="12">
         <f>F33/F34</f>
-        <v>588023.88223716291</v>
+        <v>580793.18915861798</v>
       </c>
       <c r="G35" s="12">
         <f>G33/G34</f>
-        <v>544466.55762700259</v>
+        <v>537771.47144316486</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="25" customHeight="1">
       <c r="A36" s="1"/>
       <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
+      <c r="C36" s="26"/>
+      <c r="D36" s="26"/>
+      <c r="E36" s="26"/>
+      <c r="F36" s="26"/>
+      <c r="G36" s="26"/>
     </row>
     <row r="37" spans="1:7" ht="25" customHeight="1">
       <c r="A37" s="1"/>
@@ -1478,7 +1486,10 @@
       <c r="B10" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="15"/>
+      <c r="C10" s="15">
+        <f>C6+C7*C8*C9</f>
+        <v>0.11</v>
+      </c>
       <c r="D10" s="15"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -1573,23 +1584,23 @@
       </c>
       <c r="C15" s="3">
         <f>C13*$C$10</f>
-        <v>0</v>
+        <v>132000</v>
       </c>
       <c r="D15" s="3">
         <f>D13*$C$10</f>
-        <v>0</v>
+        <v>105600</v>
       </c>
       <c r="E15" s="3">
         <f>E13*$C$10</f>
-        <v>0</v>
+        <v>79200</v>
       </c>
       <c r="F15" s="3">
         <f>F13*$C$10</f>
-        <v>0</v>
+        <v>52800</v>
       </c>
       <c r="G15" s="3">
         <f>G13*$C$10</f>
-        <v>0</v>
+        <v>26400</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="25" customHeight="1">
@@ -1599,23 +1610,23 @@
       </c>
       <c r="C16" s="3">
         <f>C14+C15</f>
-        <v>240000</v>
+        <v>372000</v>
       </c>
       <c r="D16" s="3">
         <f>D14+D15</f>
-        <v>240000</v>
+        <v>345600</v>
       </c>
       <c r="E16" s="3">
         <f>E14+E15</f>
-        <v>240000</v>
+        <v>319200</v>
       </c>
       <c r="F16" s="3">
         <f>F14+F15</f>
-        <v>240000</v>
+        <v>292800</v>
       </c>
       <c r="G16" s="3">
         <f>G14+G15</f>
-        <v>240000</v>
+        <v>266400</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="25" customHeight="1">
@@ -1660,23 +1671,23 @@
       </c>
       <c r="C19" s="17">
         <f>Proyecto!C31</f>
-        <v>832000.00000000047</v>
+        <v>828000.00000000047</v>
       </c>
       <c r="D19" s="17">
         <f>Proyecto!D31</f>
-        <v>865280.00000000093</v>
+        <v>854640.00000000093</v>
       </c>
       <c r="E19" s="17">
         <f>Proyecto!E31</f>
-        <v>899891.20000000135</v>
+        <v>888825.60000000102</v>
       </c>
       <c r="F19" s="17">
         <f>Proyecto!F31</f>
-        <v>935886.84800000093</v>
+        <v>924378.624000001</v>
       </c>
       <c r="G19" s="17">
         <f>Proyecto!G31</f>
-        <v>973322.32192000095</v>
+        <v>961353.76896000141</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="25" customHeight="1">
@@ -1686,23 +1697,23 @@
       </c>
       <c r="C20" s="16">
         <f>IF(C16=0,"Sin deuda",C19/C16)</f>
-        <v>3.4666666666666686</v>
+        <v>2.2258064516129044</v>
       </c>
       <c r="D20" s="16">
         <f>IF(D16=0,"Sin deuda",D19/D16)</f>
-        <v>3.6053333333333373</v>
+        <v>2.4729166666666695</v>
       </c>
       <c r="E20" s="16">
         <f>IF(E16=0,"Sin deuda",E19/E16)</f>
-        <v>3.7495466666666721</v>
+        <v>2.784541353383462</v>
       </c>
       <c r="F20" s="16">
         <f>IF(F16=0,"Sin deuda",F19/F16)</f>
-        <v>3.8995285333333372</v>
+        <v>3.1570308196721344</v>
       </c>
       <c r="G20" s="16">
         <f>IF(G16=0,"Sin deuda",G19/G16)</f>
-        <v>4.0555096746666708</v>
+        <v>3.6086853189189241</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="25" customHeight="1">
@@ -1712,23 +1723,23 @@
       </c>
       <c r="C21" s="3">
         <f>C19-C16</f>
-        <v>592000.00000000047</v>
+        <v>456000.00000000047</v>
       </c>
       <c r="D21" s="3">
         <f>D19-D16</f>
-        <v>625280.00000000093</v>
+        <v>509040.00000000093</v>
       </c>
       <c r="E21" s="3">
         <f>E19-E16</f>
-        <v>659891.20000000135</v>
+        <v>569625.60000000102</v>
       </c>
       <c r="F21" s="3">
         <f>F19-F16</f>
-        <v>695886.84800000093</v>
+        <v>631578.624000001</v>
       </c>
       <c r="G21" s="3">
         <f>G19-G16</f>
-        <v>733322.32192000095</v>
+        <v>694953.76896000141</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="25" customHeight="1">
@@ -1876,8 +1887,8 @@
     </row>
     <row r="4" spans="1:7" ht="25" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="2" t="s">
-        <v>56</v>
+      <c r="B4" s="2" t="str">
+        <v>Trabajo individual: 45 minutos + discusión.</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -1966,8 +1977,8 @@
     </row>
     <row r="13" spans="1:7" ht="29" customHeight="1">
       <c r="A13" s="1"/>
-      <c r="B13" s="4" t="s">
-        <v>61</v>
+      <c r="B13" s="4" t="str">
+        <v>Registro individual</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>62</v>

</xml_diff>